<commit_message>
fix: refine report presentation exports and agent pagination
</commit_message>
<xml_diff>
--- a/docs/assets/cases/auto-rules.xlsx
+++ b/docs/assets/cases/auto-rules.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1072" uniqueCount="238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1073" uniqueCount="239">
   <si>
     <t>status</t>
   </si>
@@ -158,7 +158,7 @@
     <t>["MarsCombinationRuleGenerator"]</t>
   </si>
   <si>
-    <t>0.05705639999359846</t>
+    <t>0.08245650000026217</t>
   </si>
   <si>
     <t>{"profile": "production", "direction": "high_risk", "candidate_filter": {"conditions": [{"metric": "lift", "operator": "&gt;=", "value": 1.2}, {"metric": "event_count", "operator": "&gt;=", "value": 3.0}, {"metric": "coverage", "operator": "&gt;=", "value": 0.01}, {"metric": "coverage", "operator": "&lt;=", "value": 0.5}], "targets": "primary", "target_scope": "all", "slice_pass_rate": null}, "validation_filter": {"conditions": [{"metric": "lift", "operator": "&gt;=", "value": 2.0}, {"metric": "event_count", "operator": "&gt;=", "value": 3.0}, {"metric": "coverage", "operator": "&gt;=", "value": 0.01}, {"metric": "coverage", "operator": "&lt;=", "value": 0.5}], "targets": "primary", "target_scope": "all", "slice_pass_rate": 0.8}, "grade_filters": {}, "selection_strategy": "ranked", "top_k": 5, "max_candidates": 24, "iou_threshold": 0.3, "batch_size": 100, "iou_batch_size": 512, "max_rounds": 10, "random_state": 42, "on_generator_error": "raise", "confidence_level": 0.95, "max_fdr": 0.05, "min_time_slices": 3}</t>
@@ -551,12 +551,15 @@
     <t>display_name</t>
   </si>
   <si>
+    <t>dtype</t>
+  </si>
+  <si>
+    <t>data_source</t>
+  </si>
+  <si>
     <t>description</t>
   </si>
   <si>
-    <t>data_source</t>
-  </si>
-  <si>
     <t>unit</t>
   </si>
   <si>
@@ -566,12 +569,12 @@
     <t>外部来源分 3</t>
   </si>
   <si>
+    <t>Home Credit 2018 application_{train|test}.csv</t>
+  </si>
+  <si>
     <t>Normalized score from external data source</t>
   </si>
   <si>
-    <t>Home Credit 2018 application_{train|test}.csv</t>
-  </si>
-  <si>
     <t>归一化值（无量纲）</t>
   </si>
   <si>
@@ -704,7 +707,7 @@
     <t>default_ai_queries</t>
   </si>
   <si>
-    <t>"0013ce10-ed61-4760-b773-17739bc746f1"</t>
+    <t>"56bb67a8-af4b-470b-bf3c-00cb151dca69"</t>
   </si>
   <si>
     <t>"rule"</t>
@@ -719,7 +722,7 @@
     <t>loat64","unit":"dimensionless","meaning":"规则 Wilson 事件率上界 / 同范围总体事件率；保守 Lift 上界","null":"unavailable; inspect status and report parameters"},"p_value":{"dtype":"Float64","unit":"probability","meaning":"按 direction 的单侧事件富集检验 p 值；方法见 evaluator","null":"unavailable; inspect status and report parameters"},"q_value":{"dtype":"Float64","unit":"probability","meaning":"同数据范围、target、slice、group 候选检验族 BH 校正 q 值","null":"unavailable; inspect status and report parameters"},"qualification":{"dtype":"String","unit":"state","meaning":"计算时 RuleSet 资格；快照恢复不会重建部署资格","null":"unavailable; inspect status and report parameters"},"amount_total":{"dtype":"Float64","unit":"unknown_business_unit","meaning":"当前范围已表现样本金金额和；amount_col 未提供则 null；币种见 business_context","null":"unavailable; inspect status and report parameters"},"amount_event_rate":{"dtype":"Float64","unit":"ratio","meaning":"event_amount / amount_total；零分母 null","null":"unavailable; inspect status and report parameters"},"customer_count":{"dtype":"Null","unit":"count","meaning":"当前已表现范围去重客户数；customer_col 未提供则 null","null":"unavailable; inspect status and report parameters"},"customer_event_rate":{"dtype":"Null","unit":"ratio","meaning":"event_customer_count / customer_count；不可跨规则相加","null":"unavailable; inspect status and report parameters"},"explanation":{"dtype":"String","unit":"text","meaning":"当前行所引用验证范围的中文说明；缺指标显示 N/A","null":"unavailable; inspect status and report parameters"}},"state":"computed","feature_relation":{"table":"rule_features","key":"rule_id","feature":"feature","roles":{"rule_id":"规范 DSL 的稳定哈希 ID；同 ID 可出现在不同 dataset、target 或轮次"}},"feature_query":"relation"},"rule_features":{"rows":40,"grain":"distinct rule_id / English feature; includes rejected candidates","schema_version":1,"fields":{"rule_id":{"dtype":"String","unit":"identifier","meaning":"规范 DSL 的稳定哈希 ID；同 ID 可出现在不同 dataset、target 或轮次","null":"unavailable; inspect status and report parameters"},"feature":{"dtype":"String","unit":"identifier","meaning":"AST 提取的英文输入特征 ID；中文名不替代此身份","null":"unavailable; inspect status and report parameters"}},"feature_roles":{"feature":"feature"},"state":"computed","feature_query":"direct"}}</t>
   </si>
   <si>
-    <t>{"mars_version":"0.0.28","source_project":"deimos-rule","source_commit":"e6714c5e795054e44f0c58ad7097668b4117b4a2","target":"TARGET","aux_targets":[],"features":["EXT_SOURCE_2","EXT_SOURCE_3"],"validation_status":"independent","profile":"production","qualification":"validated","group_col":null,"time_col":null,"time_grain":null,"amount_col":"AMT_CREDIT","customer_col":null,"generation_errors":[],"generator_diagnostics":[],"generators":["MarsCombinationRuleGenerator"],"elapsed_seconds":0.05705639999359846,"resolved_spec":{"profile":"production","direction":"high_risk","candidate_filter":{"conditions":[{"metric":"lift","operator":"&gt;=","value":1.2},{"metric":"event_count","operator":"&gt;=","value":3.0},{"metric":"coverage","operator":"&gt;=","value":0.01},{"metric":"coverage","operator":"&lt;=","value":0.5}],"targets":"primary","target_scope":"all","slice_pass_rate":null},"validation_filter":{"conditions":[{"metric":"lift","operator":"&gt;=","value":2.0},{"metric":"event_count","operator":"&gt;=","value":3.0},{"metric":"coverage","operator":"&gt;=","value":0.01},{"metric":"coverage","operator":"&lt;=","value":0.5}],"targets":"primary","target_scope":"all","slice_pass_rate":0.8},"grade_filters":{},"selection_strategy":"ranked","top_k":5,"max_candidates":24,"iou_threshold":0.3,"batch_size":100,"iou_batch_size":512,"max_rounds":10,"random_state":42,"on_generator_error":"raise","confidence_level":0.95,"max_fdr":0.05,"min_time_slices":3},"validation_summary":{"profile":"production","qualification":"validated","validation_status":"independent","confidence_level":0.95,"max_fdr":0.05,"min_time_slices":3,"selected_count":1,"temporal_assessed":false,"minimum_time_slice_count":0,"minimum_time_slice_pass_rate":null},"slice_definition":{"kind":"not_computed","column":null,"group_precedes_time":true,"overall_value":"__overall__"},"analysis_states":{"slices":"not_computed","interactions":"not_computed","cumulative":"not_computed","bootstrap":"not_computed"},"advanced_analysis":null}</t>
+    <t>{"mars_version":"0.0.28","source_project":"deimos-rule","source_commit":"e6714c5e795054e44f0c58ad7097668b4117b4a2","target":"TARGET","aux_targets":[],"features":["EXT_SOURCE_2","EXT_SOURCE_3"],"validation_status":"independent","profile":"production","qualification":"validated","group_col":null,"time_col":null,"time_grain":null,"amount_col":"AMT_CREDIT","customer_col":null,"generation_errors":[],"generator_diagnostics":[],"generators":["MarsCombinationRuleGenerator"],"elapsed_seconds":0.08245650000026217,"resolved_spec":{"profile":"production","direction":"high_risk","candidate_filter":{"conditions":[{"metric":"lift","operator":"&gt;=","value":1.2},{"metric":"event_count","operator":"&gt;=","value":3.0},{"metric":"coverage","operator":"&gt;=","value":0.01},{"metric":"coverage","operator":"&lt;=","value":0.5}],"targets":"primary","target_scope":"all","slice_pass_rate":null},"validation_filter":{"conditions":[{"metric":"lift","operator":"&gt;=","value":2.0},{"metric":"event_count","operator":"&gt;=","value":3.0},{"metric":"coverage","operator":"&gt;=","value":0.01},{"metric":"coverage","operator":"&lt;=","value":0.5}],"targets":"primary","target_scope":"all","slice_pass_rate":0.8},"grade_filters":{},"selection_strategy":"ranked","top_k":5,"max_candidates":24,"iou_threshold":0.3,"batch_size":100,"iou_batch_size":512,"max_rounds":10,"random_state":42,"on_generator_error":"raise","confidence_level":0.95,"max_fdr":0.05,"min_time_slices":3},"validation_summary":{"profile":"production","qualification":"validated","validation_status":"independent","confidence_level":0.95,"max_fdr":0.05,"min_time_slices":3,"selected_count":1,"temporal_assessed":false,"minimum_time_slice_count":0,"minimum_time_slice_pass_rate":null},"slice_definition":{"kind":"not_computed","column":null,"group_precedes_time":true,"overall_value":"__overall__"},"analysis_states":{"slices":"not_computed","interactions":"not_computed","cumulative":"not_computed","bootstrap":"not_computed"},"advanced_analysis":null}</t>
   </si>
   <si>
     <t>{"dataset_id":"home-credit-default-risk-2018","computation":"rule","producer":"mars.rule.MarsRuleReport","mars_version":"0.0.28","origin_project":"deimos-rule"}</t>
@@ -1130,18 +1133,18 @@
         <v>11</v>
       </c>
       <c r="C1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="D1" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B2" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C2">
         <v>1</v>
@@ -1152,10 +1155,10 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B3" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C3">
         <v>1</v>
@@ -1166,10 +1169,10 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B4" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C4">
         <v>1</v>
@@ -1180,10 +1183,10 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B5" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C5">
         <v>1</v>
@@ -1197,7 +1200,7 @@
         <v>52</v>
       </c>
       <c r="B6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C6">
         <v>1</v>
@@ -1208,10 +1211,10 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B7" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C7">
         <v>1</v>
@@ -1225,7 +1228,7 @@
         <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C8">
         <v>1</v>
@@ -1236,10 +1239,10 @@
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B9" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C9">
         <v>1</v>
@@ -1250,10 +1253,10 @@
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B10" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C10">
         <v>1</v>
@@ -1264,10 +1267,10 @@
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B11" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C11">
         <v>1</v>
@@ -1278,7 +1281,7 @@
     </row>
     <row r="12" spans="1:4">
       <c r="A12" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B12" t="s">
         <v>41</v>
@@ -1292,10 +1295,10 @@
     </row>
     <row r="13" spans="1:4">
       <c r="A13" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B13" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C13">
         <v>1</v>
@@ -1306,10 +1309,10 @@
     </row>
     <row r="14" spans="1:4">
       <c r="A14" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B14" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="C14">
         <v>1</v>
@@ -1320,10 +1323,10 @@
     </row>
     <row r="15" spans="1:4">
       <c r="A15" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B15" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C15">
         <v>1</v>
@@ -1337,7 +1340,7 @@
         <v>53</v>
       </c>
       <c r="B16" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C16">
         <v>1</v>
@@ -1348,10 +1351,10 @@
     </row>
     <row r="17" spans="1:4">
       <c r="A17" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B17" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C17">
         <v>1</v>
@@ -1362,10 +1365,10 @@
     </row>
     <row r="18" spans="1:4">
       <c r="A18" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B18" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C18">
         <v>1</v>
@@ -1376,10 +1379,10 @@
     </row>
     <row r="19" spans="1:4">
       <c r="A19" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B19" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C19">
         <v>1</v>
@@ -1406,18 +1409,18 @@
         <v>11</v>
       </c>
       <c r="C1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="D1" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C2">
         <v>1</v>
@@ -1428,10 +1431,10 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B3" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C3">
         <v>1</v>
@@ -1442,10 +1445,10 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B4" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C4">
         <v>1</v>
@@ -1456,10 +1459,10 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B5" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C5">
         <v>1</v>
@@ -1470,10 +1473,10 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B6" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C6">
         <v>2</v>
@@ -1484,10 +1487,10 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B7" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C7">
         <v>1</v>
@@ -1501,7 +1504,7 @@
         <v>52</v>
       </c>
       <c r="B8" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C8">
         <v>1</v>
@@ -1512,7 +1515,7 @@
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B9" t="s">
         <v>36</v>
@@ -1526,10 +1529,10 @@
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B10" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C10">
         <v>1</v>
@@ -1540,10 +1543,10 @@
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B11" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C11">
         <v>1</v>
@@ -1554,10 +1557,10 @@
     </row>
     <row r="12" spans="1:4">
       <c r="A12" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B12" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="C12">
         <v>1</v>
@@ -1568,10 +1571,10 @@
     </row>
     <row r="13" spans="1:4">
       <c r="A13" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B13" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C13">
         <v>1</v>
@@ -1582,10 +1585,10 @@
     </row>
     <row r="14" spans="1:4">
       <c r="A14" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B14" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C14">
         <v>1</v>
@@ -9816,10 +9819,10 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:6">
       <c r="A1" t="s">
         <v>171</v>
       </c>
@@ -9835,16 +9838,16 @@
       <c r="E1" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="2" spans="1:5">
+      <c r="F1" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
       <c r="A2" t="s">
         <v>173</v>
       </c>
       <c r="B2" t="s">
-        <v>178</v>
-      </c>
-      <c r="C2" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D2" t="s">
         <v>181</v>
@@ -9852,15 +9855,15 @@
       <c r="E2" t="s">
         <v>182</v>
       </c>
-    </row>
-    <row r="3" spans="1:5">
+      <c r="F2" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
       <c r="A3" t="s">
         <v>172</v>
       </c>
       <c r="B3" t="s">
-        <v>179</v>
-      </c>
-      <c r="C3" t="s">
         <v>180</v>
       </c>
       <c r="D3" t="s">
@@ -9868,6 +9871,9 @@
       </c>
       <c r="E3" t="s">
         <v>182</v>
+      </c>
+      <c r="F3" t="s">
+        <v>183</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: bound wide-table analysis allocations and preserve profiling contracts
</commit_message>
<xml_diff>
--- a/docs/assets/cases/auto-rules.xlsx
+++ b/docs/assets/cases/auto-rules.xlsx
@@ -158,7 +158,7 @@
     <t>["MarsCombinationRuleGenerator"]</t>
   </si>
   <si>
-    <t>0.08245650000026217</t>
+    <t>0.03689790004864335</t>
   </si>
   <si>
     <t>{"profile": "production", "direction": "high_risk", "candidate_filter": {"conditions": [{"metric": "lift", "operator": "&gt;=", "value": 1.2}, {"metric": "event_count", "operator": "&gt;=", "value": 3.0}, {"metric": "coverage", "operator": "&gt;=", "value": 0.01}, {"metric": "coverage", "operator": "&lt;=", "value": 0.5}], "targets": "primary", "target_scope": "all", "slice_pass_rate": null}, "validation_filter": {"conditions": [{"metric": "lift", "operator": "&gt;=", "value": 2.0}, {"metric": "event_count", "operator": "&gt;=", "value": 3.0}, {"metric": "coverage", "operator": "&gt;=", "value": 0.01}, {"metric": "coverage", "operator": "&lt;=", "value": 0.5}], "targets": "primary", "target_scope": "all", "slice_pass_rate": 0.8}, "grade_filters": {}, "selection_strategy": "ranked", "top_k": 5, "max_candidates": 24, "iou_threshold": 0.3, "batch_size": 100, "iou_batch_size": 512, "max_rounds": 10, "random_state": 42, "on_generator_error": "raise", "confidence_level": 0.95, "max_fdr": 0.05, "min_time_slices": 3}</t>
@@ -707,7 +707,7 @@
     <t>default_ai_queries</t>
   </si>
   <si>
-    <t>"56bb67a8-af4b-470b-bf3c-00cb151dca69"</t>
+    <t>"8fd0d348-dea5-40e5-841e-0832f4b9eba0"</t>
   </si>
   <si>
     <t>"rule"</t>
@@ -722,7 +722,7 @@
     <t>loat64","unit":"dimensionless","meaning":"规则 Wilson 事件率上界 / 同范围总体事件率；保守 Lift 上界","null":"unavailable; inspect status and report parameters"},"p_value":{"dtype":"Float64","unit":"probability","meaning":"按 direction 的单侧事件富集检验 p 值；方法见 evaluator","null":"unavailable; inspect status and report parameters"},"q_value":{"dtype":"Float64","unit":"probability","meaning":"同数据范围、target、slice、group 候选检验族 BH 校正 q 值","null":"unavailable; inspect status and report parameters"},"qualification":{"dtype":"String","unit":"state","meaning":"计算时 RuleSet 资格；快照恢复不会重建部署资格","null":"unavailable; inspect status and report parameters"},"amount_total":{"dtype":"Float64","unit":"unknown_business_unit","meaning":"当前范围已表现样本金金额和；amount_col 未提供则 null；币种见 business_context","null":"unavailable; inspect status and report parameters"},"amount_event_rate":{"dtype":"Float64","unit":"ratio","meaning":"event_amount / amount_total；零分母 null","null":"unavailable; inspect status and report parameters"},"customer_count":{"dtype":"Null","unit":"count","meaning":"当前已表现范围去重客户数；customer_col 未提供则 null","null":"unavailable; inspect status and report parameters"},"customer_event_rate":{"dtype":"Null","unit":"ratio","meaning":"event_customer_count / customer_count；不可跨规则相加","null":"unavailable; inspect status and report parameters"},"explanation":{"dtype":"String","unit":"text","meaning":"当前行所引用验证范围的中文说明；缺指标显示 N/A","null":"unavailable; inspect status and report parameters"}},"state":"computed","feature_relation":{"table":"rule_features","key":"rule_id","feature":"feature","roles":{"rule_id":"规范 DSL 的稳定哈希 ID；同 ID 可出现在不同 dataset、target 或轮次"}},"feature_query":"relation"},"rule_features":{"rows":40,"grain":"distinct rule_id / English feature; includes rejected candidates","schema_version":1,"fields":{"rule_id":{"dtype":"String","unit":"identifier","meaning":"规范 DSL 的稳定哈希 ID；同 ID 可出现在不同 dataset、target 或轮次","null":"unavailable; inspect status and report parameters"},"feature":{"dtype":"String","unit":"identifier","meaning":"AST 提取的英文输入特征 ID；中文名不替代此身份","null":"unavailable; inspect status and report parameters"}},"feature_roles":{"feature":"feature"},"state":"computed","feature_query":"direct"}}</t>
   </si>
   <si>
-    <t>{"mars_version":"0.0.28","source_project":"deimos-rule","source_commit":"e6714c5e795054e44f0c58ad7097668b4117b4a2","target":"TARGET","aux_targets":[],"features":["EXT_SOURCE_2","EXT_SOURCE_3"],"validation_status":"independent","profile":"production","qualification":"validated","group_col":null,"time_col":null,"time_grain":null,"amount_col":"AMT_CREDIT","customer_col":null,"generation_errors":[],"generator_diagnostics":[],"generators":["MarsCombinationRuleGenerator"],"elapsed_seconds":0.08245650000026217,"resolved_spec":{"profile":"production","direction":"high_risk","candidate_filter":{"conditions":[{"metric":"lift","operator":"&gt;=","value":1.2},{"metric":"event_count","operator":"&gt;=","value":3.0},{"metric":"coverage","operator":"&gt;=","value":0.01},{"metric":"coverage","operator":"&lt;=","value":0.5}],"targets":"primary","target_scope":"all","slice_pass_rate":null},"validation_filter":{"conditions":[{"metric":"lift","operator":"&gt;=","value":2.0},{"metric":"event_count","operator":"&gt;=","value":3.0},{"metric":"coverage","operator":"&gt;=","value":0.01},{"metric":"coverage","operator":"&lt;=","value":0.5}],"targets":"primary","target_scope":"all","slice_pass_rate":0.8},"grade_filters":{},"selection_strategy":"ranked","top_k":5,"max_candidates":24,"iou_threshold":0.3,"batch_size":100,"iou_batch_size":512,"max_rounds":10,"random_state":42,"on_generator_error":"raise","confidence_level":0.95,"max_fdr":0.05,"min_time_slices":3},"validation_summary":{"profile":"production","qualification":"validated","validation_status":"independent","confidence_level":0.95,"max_fdr":0.05,"min_time_slices":3,"selected_count":1,"temporal_assessed":false,"minimum_time_slice_count":0,"minimum_time_slice_pass_rate":null},"slice_definition":{"kind":"not_computed","column":null,"group_precedes_time":true,"overall_value":"__overall__"},"analysis_states":{"slices":"not_computed","interactions":"not_computed","cumulative":"not_computed","bootstrap":"not_computed"},"advanced_analysis":null}</t>
+    <t>{"mars_version":"0.0.28","source_project":"deimos-rule","source_commit":"e6714c5e795054e44f0c58ad7097668b4117b4a2","target":"TARGET","aux_targets":[],"features":["EXT_SOURCE_2","EXT_SOURCE_3"],"validation_status":"independent","profile":"production","qualification":"validated","group_col":null,"time_col":null,"time_grain":null,"amount_col":"AMT_CREDIT","customer_col":null,"generation_errors":[],"generator_diagnostics":[],"generators":["MarsCombinationRuleGenerator"],"elapsed_seconds":0.03689790004864335,"resolved_spec":{"profile":"production","direction":"high_risk","candidate_filter":{"conditions":[{"metric":"lift","operator":"&gt;=","value":1.2},{"metric":"event_count","operator":"&gt;=","value":3.0},{"metric":"coverage","operator":"&gt;=","value":0.01},{"metric":"coverage","operator":"&lt;=","value":0.5}],"targets":"primary","target_scope":"all","slice_pass_rate":null},"validation_filter":{"conditions":[{"metric":"lift","operator":"&gt;=","value":2.0},{"metric":"event_count","operator":"&gt;=","value":3.0},{"metric":"coverage","operator":"&gt;=","value":0.01},{"metric":"coverage","operator":"&lt;=","value":0.5}],"targets":"primary","target_scope":"all","slice_pass_rate":0.8},"grade_filters":{},"selection_strategy":"ranked","top_k":5,"max_candidates":24,"iou_threshold":0.3,"batch_size":100,"iou_batch_size":512,"max_rounds":10,"random_state":42,"on_generator_error":"raise","confidence_level":0.95,"max_fdr":0.05,"min_time_slices":3},"validation_summary":{"profile":"production","qualification":"validated","validation_status":"independent","confidence_level":0.95,"max_fdr":0.05,"min_time_slices":3,"selected_count":1,"temporal_assessed":false,"minimum_time_slice_count":0,"minimum_time_slice_pass_rate":null},"slice_definition":{"kind":"not_computed","column":null,"group_precedes_time":true,"overall_value":"__overall__"},"analysis_states":{"slices":"not_computed","interactions":"not_computed","cumulative":"not_computed","bootstrap":"not_computed"},"advanced_analysis":null}</t>
   </si>
   <si>
     <t>{"dataset_id":"home-credit-default-risk-2018","computation":"rule","producer":"mars.rule.MarsRuleReport","mars_version":"0.0.28","origin_project":"deimos-rule"}</t>

</xml_diff>

<commit_message>
fix: preserve streaming row alignment and enforce capacity evidence
</commit_message>
<xml_diff>
--- a/docs/assets/cases/auto-rules.xlsx
+++ b/docs/assets/cases/auto-rules.xlsx
@@ -158,7 +158,7 @@
     <t>["MarsCombinationRuleGenerator"]</t>
   </si>
   <si>
-    <t>0.03689790004864335</t>
+    <t>0.03716130007524043</t>
   </si>
   <si>
     <t>{"profile": "production", "direction": "high_risk", "candidate_filter": {"conditions": [{"metric": "lift", "operator": "&gt;=", "value": 1.2}, {"metric": "event_count", "operator": "&gt;=", "value": 3.0}, {"metric": "coverage", "operator": "&gt;=", "value": 0.01}, {"metric": "coverage", "operator": "&lt;=", "value": 0.5}], "targets": "primary", "target_scope": "all", "slice_pass_rate": null}, "validation_filter": {"conditions": [{"metric": "lift", "operator": "&gt;=", "value": 2.0}, {"metric": "event_count", "operator": "&gt;=", "value": 3.0}, {"metric": "coverage", "operator": "&gt;=", "value": 0.01}, {"metric": "coverage", "operator": "&lt;=", "value": 0.5}], "targets": "primary", "target_scope": "all", "slice_pass_rate": 0.8}, "grade_filters": {}, "selection_strategy": "ranked", "top_k": 5, "max_candidates": 24, "iou_threshold": 0.3, "batch_size": 100, "iou_batch_size": 512, "max_rounds": 10, "random_state": 42, "on_generator_error": "raise", "confidence_level": 0.95, "max_fdr": 0.05, "min_time_slices": 3}</t>
@@ -707,7 +707,7 @@
     <t>default_ai_queries</t>
   </si>
   <si>
-    <t>"8fd0d348-dea5-40e5-841e-0832f4b9eba0"</t>
+    <t>"4da17b8e-8213-4cf5-8018-102ace5b41e5"</t>
   </si>
   <si>
     <t>"rule"</t>
@@ -722,7 +722,7 @@
     <t>loat64","unit":"dimensionless","meaning":"规则 Wilson 事件率上界 / 同范围总体事件率；保守 Lift 上界","null":"unavailable; inspect status and report parameters"},"p_value":{"dtype":"Float64","unit":"probability","meaning":"按 direction 的单侧事件富集检验 p 值；方法见 evaluator","null":"unavailable; inspect status and report parameters"},"q_value":{"dtype":"Float64","unit":"probability","meaning":"同数据范围、target、slice、group 候选检验族 BH 校正 q 值","null":"unavailable; inspect status and report parameters"},"qualification":{"dtype":"String","unit":"state","meaning":"计算时 RuleSet 资格；快照恢复不会重建部署资格","null":"unavailable; inspect status and report parameters"},"amount_total":{"dtype":"Float64","unit":"unknown_business_unit","meaning":"当前范围已表现样本金金额和；amount_col 未提供则 null；币种见 business_context","null":"unavailable; inspect status and report parameters"},"amount_event_rate":{"dtype":"Float64","unit":"ratio","meaning":"event_amount / amount_total；零分母 null","null":"unavailable; inspect status and report parameters"},"customer_count":{"dtype":"Null","unit":"count","meaning":"当前已表现范围去重客户数；customer_col 未提供则 null","null":"unavailable; inspect status and report parameters"},"customer_event_rate":{"dtype":"Null","unit":"ratio","meaning":"event_customer_count / customer_count；不可跨规则相加","null":"unavailable; inspect status and report parameters"},"explanation":{"dtype":"String","unit":"text","meaning":"当前行所引用验证范围的中文说明；缺指标显示 N/A","null":"unavailable; inspect status and report parameters"}},"state":"computed","feature_relation":{"table":"rule_features","key":"rule_id","feature":"feature","roles":{"rule_id":"规范 DSL 的稳定哈希 ID；同 ID 可出现在不同 dataset、target 或轮次"}},"feature_query":"relation"},"rule_features":{"rows":40,"grain":"distinct rule_id / English feature; includes rejected candidates","schema_version":1,"fields":{"rule_id":{"dtype":"String","unit":"identifier","meaning":"规范 DSL 的稳定哈希 ID；同 ID 可出现在不同 dataset、target 或轮次","null":"unavailable; inspect status and report parameters"},"feature":{"dtype":"String","unit":"identifier","meaning":"AST 提取的英文输入特征 ID；中文名不替代此身份","null":"unavailable; inspect status and report parameters"}},"feature_roles":{"feature":"feature"},"state":"computed","feature_query":"direct"}}</t>
   </si>
   <si>
-    <t>{"mars_version":"0.0.28","source_project":"deimos-rule","source_commit":"e6714c5e795054e44f0c58ad7097668b4117b4a2","target":"TARGET","aux_targets":[],"features":["EXT_SOURCE_2","EXT_SOURCE_3"],"validation_status":"independent","profile":"production","qualification":"validated","group_col":null,"time_col":null,"time_grain":null,"amount_col":"AMT_CREDIT","customer_col":null,"generation_errors":[],"generator_diagnostics":[],"generators":["MarsCombinationRuleGenerator"],"elapsed_seconds":0.03689790004864335,"resolved_spec":{"profile":"production","direction":"high_risk","candidate_filter":{"conditions":[{"metric":"lift","operator":"&gt;=","value":1.2},{"metric":"event_count","operator":"&gt;=","value":3.0},{"metric":"coverage","operator":"&gt;=","value":0.01},{"metric":"coverage","operator":"&lt;=","value":0.5}],"targets":"primary","target_scope":"all","slice_pass_rate":null},"validation_filter":{"conditions":[{"metric":"lift","operator":"&gt;=","value":2.0},{"metric":"event_count","operator":"&gt;=","value":3.0},{"metric":"coverage","operator":"&gt;=","value":0.01},{"metric":"coverage","operator":"&lt;=","value":0.5}],"targets":"primary","target_scope":"all","slice_pass_rate":0.8},"grade_filters":{},"selection_strategy":"ranked","top_k":5,"max_candidates":24,"iou_threshold":0.3,"batch_size":100,"iou_batch_size":512,"max_rounds":10,"random_state":42,"on_generator_error":"raise","confidence_level":0.95,"max_fdr":0.05,"min_time_slices":3},"validation_summary":{"profile":"production","qualification":"validated","validation_status":"independent","confidence_level":0.95,"max_fdr":0.05,"min_time_slices":3,"selected_count":1,"temporal_assessed":false,"minimum_time_slice_count":0,"minimum_time_slice_pass_rate":null},"slice_definition":{"kind":"not_computed","column":null,"group_precedes_time":true,"overall_value":"__overall__"},"analysis_states":{"slices":"not_computed","interactions":"not_computed","cumulative":"not_computed","bootstrap":"not_computed"},"advanced_analysis":null}</t>
+    <t>{"mars_version":"0.0.28","source_project":"deimos-rule","source_commit":"e6714c5e795054e44f0c58ad7097668b4117b4a2","target":"TARGET","aux_targets":[],"features":["EXT_SOURCE_2","EXT_SOURCE_3"],"validation_status":"independent","profile":"production","qualification":"validated","group_col":null,"time_col":null,"time_grain":null,"amount_col":"AMT_CREDIT","customer_col":null,"generation_errors":[],"generator_diagnostics":[],"generators":["MarsCombinationRuleGenerator"],"elapsed_seconds":0.03716130007524043,"resolved_spec":{"profile":"production","direction":"high_risk","candidate_filter":{"conditions":[{"metric":"lift","operator":"&gt;=","value":1.2},{"metric":"event_count","operator":"&gt;=","value":3.0},{"metric":"coverage","operator":"&gt;=","value":0.01},{"metric":"coverage","operator":"&lt;=","value":0.5}],"targets":"primary","target_scope":"all","slice_pass_rate":null},"validation_filter":{"conditions":[{"metric":"lift","operator":"&gt;=","value":2.0},{"metric":"event_count","operator":"&gt;=","value":3.0},{"metric":"coverage","operator":"&gt;=","value":0.01},{"metric":"coverage","operator":"&lt;=","value":0.5}],"targets":"primary","target_scope":"all","slice_pass_rate":0.8},"grade_filters":{},"selection_strategy":"ranked","top_k":5,"max_candidates":24,"iou_threshold":0.3,"batch_size":100,"iou_batch_size":512,"max_rounds":10,"random_state":42,"on_generator_error":"raise","confidence_level":0.95,"max_fdr":0.05,"min_time_slices":3},"validation_summary":{"profile":"production","qualification":"validated","validation_status":"independent","confidence_level":0.95,"max_fdr":0.05,"min_time_slices":3,"selected_count":1,"temporal_assessed":false,"minimum_time_slice_count":0,"minimum_time_slice_pass_rate":null},"slice_definition":{"kind":"not_computed","column":null,"group_precedes_time":true,"overall_value":"__overall__"},"analysis_states":{"slices":"not_computed","interactions":"not_computed","cumulative":"not_computed","bootstrap":"not_computed"},"advanced_analysis":null}</t>
   </si>
   <si>
     <t>{"dataset_id":"home-credit-default-risk-2018","computation":"rule","producer":"mars.rule.MarsRuleReport","mars_version":"0.0.28","origin_project":"deimos-rule"}</t>

</xml_diff>